<commit_message>
add: create & read playlist (fe be) | todo: update, delete, design, layout
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232CD508-94F5-41C0-BABE-6AF13BD505E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A19316-99C1-40AF-9926-4D00AB0338E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="2" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>40.297361856224668</v>
+        <v>41.619430821741915</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -8183,11 +8183,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="121">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="65">
         <f t="shared" ref="F6:F12" ca="1" si="1">E6/4*C6</f>
-        <v>0</v>
+        <v>6.2068965517241378E-2</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -8203,11 +8203,11 @@
         <v>2</v>
       </c>
       <c r="E7" s="123">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.12413793103448276</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -8253,17 +8253,17 @@
       </c>
       <c r="E9" s="74">
         <f>(H9/J9*4)-((1-I9)*(H9/J9*2))</f>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.19862068965517243</v>
       </c>
       <c r="H9" s="138">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I9" s="138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="136">
         <v>10</v>
@@ -8282,11 +8282,11 @@
         <v>1</v>
       </c>
       <c r="E10" s="124">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>6.2068965517241378E-2</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -8342,11 +8342,11 @@
         <v>8</v>
       </c>
       <c r="E13" s="124">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F13" s="65">
         <f ca="1">E13/4*C13</f>
-        <v>0</v>
+        <v>0.49655172413793103</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -8405,7 +8405,7 @@
       <c r="E16" s="52"/>
       <c r="F16" s="62">
         <f ca="1">SUM(F6:F15)</f>
-        <v>0</v>
+        <v>0.94344827586206903</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" thickTop="1">
@@ -8458,11 +8458,11 @@
         <v>2</v>
       </c>
       <c r="E20" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20" s="25">
         <f ca="1">E20/4 * C20</f>
-        <v>0</v>
+        <v>3.0000000000000006E-2</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -8478,11 +8478,11 @@
         <v>3</v>
       </c>
       <c r="E21" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="25">
         <f ca="1">E21/4 * C21</f>
-        <v>0</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -8498,11 +8498,11 @@
         <v>3</v>
       </c>
       <c r="E22" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22" s="25">
         <f ca="1">E22/4 * C22</f>
-        <v>0</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -8518,11 +8518,11 @@
         <v>1</v>
       </c>
       <c r="E23" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23" s="25">
         <f ca="1">E23/4 * C23</f>
-        <v>0</v>
+        <v>1.5000000000000003E-2</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -8538,11 +8538,11 @@
         <v>1</v>
       </c>
       <c r="E24" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24" s="25">
         <f ca="1">E24/4 * C24</f>
-        <v>0</v>
+        <v>1.5000000000000003E-2</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
@@ -8560,7 +8560,7 @@
       <c r="E25" s="35"/>
       <c r="F25" s="34">
         <f ca="1">SUM(F20:F24)</f>
-        <v>0</v>
+        <v>0.15000000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -8573,7 +8573,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F16,F25)</f>
-        <v>0</v>
+        <v>1.0934482758620692</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -9725,17 +9725,17 @@
       </c>
       <c r="E9" s="74">
         <f>(H9/J9*4)-((1-I9)*(H9/J9*2))</f>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.19862068965517243</v>
       </c>
       <c r="H9" s="138">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I9" s="138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="136">
         <v>10</v>
@@ -9870,7 +9870,7 @@
       <c r="E16" s="52"/>
       <c r="F16" s="62">
         <f ca="1">SUM(F6:F15)</f>
-        <v>0.74482758620689649</v>
+        <v>0.94344827586206903</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="15.75" thickTop="1"/>
@@ -10029,7 +10029,7 @@
       <c r="E27" s="221"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F16,F25)</f>
-        <v>0.94482758620689644</v>
+        <v>1.143448275862069</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13078,11 +13078,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="65">
         <f ca="1">E6/4*C6</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -13301,7 +13301,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13450,7 +13450,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23336,11 +23336,11 @@
       </c>
       <c r="D22" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.54672413793103458</v>
       </c>
       <c r="E22" s="40">
         <f ca="1">'Following Page'!F27</f>
-        <v>0</v>
+        <v>1.0934482758620692</v>
       </c>
     </row>
     <row r="23" spans="2:8">
@@ -23352,11 +23352,11 @@
       </c>
       <c r="D23" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.47241379310344822</v>
+        <v>0.57172413793103449</v>
       </c>
       <c r="E23" s="40">
         <f ca="1">'Friends Page'!F27</f>
-        <v>0.94482758620689644</v>
+        <v>1.143448275862069</v>
       </c>
     </row>
     <row r="24" spans="2:8">
@@ -23384,11 +23384,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23613,7 +23613,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>40.297361856224668</v>
+        <v>41.619430821741915</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23623,7 +23623,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.40297361856224667</v>
+        <v>0.41619430821741915</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23634,7 +23634,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>40.297361856224668</v>
+        <v>41.619430821741915</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51520,6 +51520,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51742,16 +51751,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51770,14 +51778,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: playlist page styling, update, delete, reorder by dnd
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A19316-99C1-40AF-9926-4D00AB0338E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76060C29-8B87-4E50-90F6-A8C2E7CA77A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="2" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>41.619430821741915</v>
+        <v>43.106573678884764</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -13118,11 +13118,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ref="F8:F16" ca="1" si="2">E8/4*C8</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -13138,11 +13138,11 @@
         <v>3</v>
       </c>
       <c r="E9" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.18000000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -13158,11 +13158,11 @@
         <v>3</v>
       </c>
       <c r="E10" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.18000000000000002</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -13178,11 +13178,11 @@
         <v>5</v>
       </c>
       <c r="E11" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -13198,11 +13198,11 @@
         <v>5</v>
       </c>
       <c r="E12" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -13238,11 +13238,11 @@
         <v>4</v>
       </c>
       <c r="E14" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -13278,11 +13278,11 @@
         <v>2</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" thickBot="1">
@@ -13301,7 +13301,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>0.03</v>
+        <v>1.4100000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13354,11 +13354,11 @@
         <v>2</v>
       </c>
       <c r="E21" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="25">
         <f ca="1">E21/4 * C21</f>
-        <v>0</v>
+        <v>4.2857142857142858E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -13374,11 +13374,11 @@
         <v>3</v>
       </c>
       <c r="E22" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22" s="25">
         <f ca="1">E22/4 * C22</f>
-        <v>0</v>
+        <v>6.4285714285714279E-2</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -13437,7 +13437,7 @@
       <c r="E25" s="35"/>
       <c r="F25" s="34">
         <f ca="1">SUM(F21:F24)</f>
-        <v>0</v>
+        <v>0.10714285714285714</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13450,7 +13450,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>0.03</v>
+        <v>1.5171428571428573</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23384,11 +23384,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>0.75857142857142867</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>0.03</v>
+        <v>1.5171428571428573</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23613,7 +23613,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>41.619430821741915</v>
+        <v>43.106573678884764</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23623,7 +23623,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.41619430821741915</v>
+        <v>0.43106573678884763</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23634,7 +23634,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>41.619430821741915</v>
+        <v>43.106573678884764</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51520,15 +51520,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51751,15 +51742,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51778,6 +51770,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: tab controls in profile page (video & playlist tab) | update: fetch video attributes from activity-service
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76060C29-8B87-4E50-90F6-A8C2E7CA77A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFB73FC-03D1-412A-A8E4-C4A4A89FB7F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="2" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>43.106573678884764</v>
+        <v>44.535729523040608</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11344,11 +11344,11 @@
         <v>1</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>4.6753246753246755E-2</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -11404,11 +11404,11 @@
         <v>3</v>
       </c>
       <c r="E19" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F19" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.14025974025974025</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -11425,14 +11425,14 @@
       </c>
       <c r="E20" s="80">
         <f>H20*4/I20</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F20" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.14025974025974025</v>
       </c>
       <c r="H20" s="138">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I20" s="136">
         <v>2</v>
@@ -11452,14 +11452,14 @@
       </c>
       <c r="E21" s="80">
         <f>H21*4/I21</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>3.5064935064935063E-2</v>
       </c>
       <c r="H21" s="138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" s="136">
         <v>4</v>
@@ -11478,11 +11478,11 @@
         <v>5</v>
       </c>
       <c r="E22" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F22" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.17532467532467533</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -11519,14 +11519,14 @@
       </c>
       <c r="E24" s="80">
         <f>H24*4/I24</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F24" s="79">
         <f t="shared" ref="F24:F25" ca="1" si="3">E24/4*C24</f>
-        <v>0</v>
+        <v>0.14025974025974025</v>
       </c>
       <c r="H24" s="138">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I24" s="136">
         <v>3</v>
@@ -11545,11 +11545,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F25" s="79">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>2.3376623376623377E-2</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -11564,7 +11564,9 @@
       <c r="D26" s="73">
         <v>2</v>
       </c>
-      <c r="E26" s="122"/>
+      <c r="E26" s="122">
+        <v>0</v>
+      </c>
       <c r="F26" s="79">
         <f t="shared" ca="1" si="1"/>
         <v>0</v>
@@ -11840,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>0.8282003710575141</v>
+        <v>1.5294990723562154</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -11999,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>1.2282003710575142</v>
+        <v>1.9294990723562155</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13098,11 +13100,11 @@
         <v>1</v>
       </c>
       <c r="E7" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f ca="1">E7/4*C7</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -13301,7 +13303,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>1.4100000000000001</v>
+        <v>1.4700000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13394,11 +13396,11 @@
         <v>1</v>
       </c>
       <c r="E23" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23" s="25">
         <f ca="1">E23/4 * C23</f>
-        <v>0</v>
+        <v>2.1428571428571429E-2</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -13414,11 +13416,11 @@
         <v>1</v>
       </c>
       <c r="E24" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24" s="25">
         <f ca="1">E24/4 * C24</f>
-        <v>0</v>
+        <v>2.1428571428571429E-2</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
@@ -13437,7 +13439,7 @@
       <c r="E25" s="35"/>
       <c r="F25" s="34">
         <f ca="1">SUM(F21:F24)</f>
-        <v>0.10714285714285714</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13450,7 +13452,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>1.5171428571428573</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -20049,11 +20051,11 @@
         <v>8</v>
       </c>
       <c r="E12" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -20212,7 +20214,7 @@
       <c r="E20" s="82"/>
       <c r="F20" s="83">
         <f ca="1">SUM(F6:F19)</f>
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" thickTop="1">
@@ -20265,11 +20267,11 @@
         <v>2</v>
       </c>
       <c r="E24" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" s="25">
         <f ca="1">E24/4 * C24</f>
-        <v>0.05</v>
+        <v>7.5000000000000011E-2</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -20285,11 +20287,11 @@
         <v>3</v>
       </c>
       <c r="E25" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" s="25">
         <f ca="1">E25/4 * C25</f>
-        <v>7.4999999999999997E-2</v>
+        <v>0.11249999999999999</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>234</v>
@@ -20308,11 +20310,11 @@
         <v>3</v>
       </c>
       <c r="E26" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" s="25">
         <f ca="1">E26/4 * C26</f>
-        <v>7.4999999999999997E-2</v>
+        <v>0.11249999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -20328,11 +20330,11 @@
         <v>1</v>
       </c>
       <c r="E27" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" s="25">
         <f ca="1">E27/4 * C27</f>
-        <v>2.5000000000000001E-2</v>
+        <v>3.7500000000000006E-2</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -20348,11 +20350,11 @@
         <v>1</v>
       </c>
       <c r="E28" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28" s="25">
         <f ca="1">E28/4 * C28</f>
-        <v>2.5000000000000001E-2</v>
+        <v>3.7500000000000006E-2</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15.75" thickBot="1">
@@ -20371,7 +20373,7 @@
       <c r="E29" s="35"/>
       <c r="F29" s="34">
         <f ca="1">SUM(F24:F28)</f>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15.75" thickTop="1">
@@ -20387,7 +20389,7 @@
       <c r="E31" s="238"/>
       <c r="F31" s="107">
         <f ca="1">SUM(F20,F29)</f>
-        <v>2</v>
+        <v>2.625</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" thickTop="1">
@@ -23368,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.30705009276437856</v>
+        <v>0.48237476808905388</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>1.2282003710575142</v>
+        <v>1.9294990723562155</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23384,11 +23386,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.75857142857142867</v>
+        <v>0.81</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>1.5171428571428573</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23464,11 +23466,11 @@
       </c>
       <c r="D30" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
       <c r="E30" s="40">
         <f ca="1">'Studio Upload Page'!F31</f>
-        <v>2</v>
+        <v>2.625</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -23613,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>43.106573678884764</v>
+        <v>44.535729523040608</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23623,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.43106573678884763</v>
+        <v>0.44535729523040607</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23634,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>43.106573678884764</v>
+        <v>44.535729523040608</v>
       </c>
       <c r="E41" s="203"/>
     </row>

</xml_diff>

<commit_message>
add: search page | fix: unauthenticated bug in useVideos.ts
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFB73FC-03D1-412A-A8E4-C4A4A89FB7F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D86CDA-8B13-44B8-8FF1-D544F2C8C16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>44.535729523040608</v>
+        <v>46.677515237326325</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -13260,11 +13260,11 @@
         <v>3</v>
       </c>
       <c r="E15" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F15" s="79">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.13500000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -13303,7 +13303,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>1.4700000000000002</v>
+        <v>1.605</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13452,7 +13452,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>1.62</v>
+        <v>1.7549999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -14541,11 +14541,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="65">
         <f ca="1">E6/4*C6</f>
-        <v>0</v>
+        <v>3.8571428571428576E-2</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -14561,11 +14561,11 @@
         <v>5</v>
       </c>
       <c r="E7" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f t="shared" ref="F7:F18" ca="1" si="1">E7/4*C7</f>
-        <v>0</v>
+        <v>0.19285714285714287</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -14601,11 +14601,11 @@
         <v>7</v>
       </c>
       <c r="E9" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -14621,11 +14621,11 @@
         <v>10</v>
       </c>
       <c r="E10" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.19285714285714287</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -14641,11 +14641,11 @@
         <v>10</v>
       </c>
       <c r="E11" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.38571428571428573</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -14661,11 +14661,11 @@
         <v>12</v>
       </c>
       <c r="E12" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.23142857142857146</v>
       </c>
       <c r="H12" s="134" t="s">
         <v>322</v>
@@ -14688,14 +14688,14 @@
       </c>
       <c r="E13" s="3">
         <f>H13*4/I13</f>
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="F13" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.23142857142857143</v>
       </c>
       <c r="H13" s="135">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I13" s="136">
         <v>10</v>
@@ -14715,14 +14715,14 @@
       </c>
       <c r="E14" s="3">
         <f>H14*4/I14</f>
-        <v>0</v>
+        <v>3.5555555555555554</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.17142857142857143</v>
       </c>
       <c r="H14" s="135">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I14" s="136">
         <v>9</v>
@@ -14741,11 +14741,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F15" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2.8928571428571432E-2</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -14761,11 +14761,11 @@
         <v>1</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>3.8571428571428576E-2</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -14824,7 +14824,7 @@
       <c r="E19" s="82"/>
       <c r="F19" s="69">
         <f ca="1">SUM(F6:F18)</f>
-        <v>0</v>
+        <v>1.7817857142857145</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.75" thickTop="1">
@@ -14877,11 +14877,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23" s="25">
         <f ca="1">E23/4 * C23</f>
-        <v>0</v>
+        <v>3.3750000000000002E-2</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -14897,11 +14897,11 @@
         <v>10</v>
       </c>
       <c r="E24" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24" s="25">
         <f ca="1">E24/4 * C24</f>
-        <v>0</v>
+        <v>2.2500000000000006E-2</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -14917,11 +14917,11 @@
         <v>15</v>
       </c>
       <c r="E25" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F25" s="25">
         <f ca="1">E25/4 * C25</f>
-        <v>0</v>
+        <v>3.3750000000000002E-2</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -14937,11 +14937,11 @@
         <v>30</v>
       </c>
       <c r="E26" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F26" s="25">
         <f ca="1">E26/4 * C26</f>
-        <v>0</v>
+        <v>6.7500000000000004E-2</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1">
@@ -14956,11 +14956,11 @@
         <v>30</v>
       </c>
       <c r="E27" s="112">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F27" s="25">
         <f ca="1">E27/4 * C27</f>
-        <v>0</v>
+        <v>6.7500000000000004E-2</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
@@ -14978,7 +14978,7 @@
       <c r="E28" s="35"/>
       <c r="F28" s="34">
         <f ca="1">SUM(F23:F27)</f>
-        <v>0</v>
+        <v>0.22500000000000003</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -14991,7 +14991,7 @@
       <c r="E30" s="238"/>
       <c r="F30" s="107">
         <f ca="1">SUM(,F19,F28)</f>
-        <v>0</v>
+        <v>2.0067857142857144</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23386,11 +23386,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.81</v>
+        <v>0.87749999999999995</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>1.62</v>
+        <v>1.7549999999999999</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23402,11 +23402,11 @@
       </c>
       <c r="D26" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.66892857142857143</v>
       </c>
       <c r="E26" s="40">
         <f ca="1">'Search Page'!F30</f>
-        <v>0</v>
+        <v>2.0067857142857144</v>
       </c>
     </row>
     <row r="27" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>44.535729523040608</v>
+        <v>46.677515237326325</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.44535729523040607</v>
+        <v>0.46677515237326328</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>44.535729523040608</v>
+        <v>46.677515237326325</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: liked videos tab in profile page
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D86CDA-8B13-44B8-8FF1-D544F2C8C16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE1B371-62E3-4E8E-9BD9-A8EB0547F582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>46.677515237326325</v>
+        <v>47.401628596601654</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11652,11 +11652,11 @@
         <v>2</v>
       </c>
       <c r="E30" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F30" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.350649350649351E-2</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -11672,11 +11672,11 @@
         <v>2</v>
       </c>
       <c r="E31" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F31" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.350649350649351E-2</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -11693,14 +11693,14 @@
       </c>
       <c r="E32" s="80">
         <f>H32*4/I32</f>
-        <v>0</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="F32" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.3506493506493496E-2</v>
       </c>
       <c r="H32" s="138">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I32" s="136">
         <v>3</v>
@@ -11719,11 +11719,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F33" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>4.6753246753246755E-2</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -11842,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>1.5294990723562154</v>
+        <v>1.8567717996289428</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -12001,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>1.9294990723562155</v>
+        <v>2.2567717996289427</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.43499551741803272</v>
+        <v>0.46240010245901647</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>5.2199462090163928</v>
+        <v>5.5488012295081974</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23370,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.48237476808905388</v>
+        <v>0.56419294990723567</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>1.9294990723562155</v>
+        <v>2.2567717996289427</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.39226618705035976</v>
+        <v>0.40197841726618699</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>2.7458633093525182</v>
+        <v>2.8138489208633088</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>46.677515237326325</v>
+        <v>47.401628596601654</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.46677515237326328</v>
+        <v>0.47401628596601653</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>46.677515237326325</v>
+        <v>47.401628596601654</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -24890,14 +24890,14 @@
       </c>
       <c r="E14" s="4">
         <f>H14/I14*4</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>6.7985611510791369E-2</v>
       </c>
       <c r="H14" s="135">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="136">
         <v>4</v>
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>2.2208633093525183</v>
+        <v>2.2888489208633089</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>2.7458633093525182</v>
+        <v>2.8138489208633088</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -43537,11 +43537,11 @@
         <v>2</v>
       </c>
       <c r="N15" s="53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O15" s="120">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>6.3281250000000011E-2</v>
       </c>
     </row>
     <row r="16" spans="2:18">
@@ -43592,11 +43592,11 @@
         <v>4</v>
       </c>
       <c r="E17" s="53">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>0.26557377049180331</v>
       </c>
       <c r="K17" s="118" t="s">
         <v>66</v>
@@ -44048,7 +44048,7 @@
       <c r="N29" s="82"/>
       <c r="O29" s="69">
         <f ca="1">SUM(O9:O28)</f>
-        <v>0.65109375000000003</v>
+        <v>0.71437499999999998</v>
       </c>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" thickTop="1">
@@ -44340,7 +44340,7 @@
       <c r="N39" s="237"/>
       <c r="O39" s="115">
         <f ca="1">SUM(O29,O37)</f>
-        <v>0.80109375000000005</v>
+        <v>0.864375</v>
       </c>
     </row>
     <row r="40" spans="2:15" ht="15.75" customHeight="1" thickTop="1">
@@ -44396,7 +44396,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>3.5188524590163932</v>
+        <v>3.7844262295081976</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44536,7 +44536,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>4.4188524590163931</v>
+        <v>4.6844262295081975</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44550,7 +44550,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>5.2199462090163928</v>
+        <v>5.5488012295081974</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: notification toast, share modal (unfinished), unsend comment/reply, message list (unfinished)
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE1B371-62E3-4E8E-9BD9-A8EB0547F582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DE47A6-9201-46DA-A0A7-CD576A68D1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="9" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>47.401628596601654</v>
+        <v>48.935046452480883</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.46240010245901647</v>
+        <v>0.56752305327868868</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>5.5488012295081974</v>
+        <v>6.8102766393442637</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.40197841726618699</v>
+        <v>0.44082733812949632</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>2.8138489208633088</v>
+        <v>3.085791366906474</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>47.401628596601654</v>
+        <v>48.935046452480883</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.47401628596601653</v>
+        <v>0.48935046452480885</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>47.401628596601654</v>
+        <v>48.935046452480883</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -24916,11 +24916,11 @@
         <v>2</v>
       </c>
       <c r="E15" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.0647482014388492E-2</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -24936,11 +24936,11 @@
         <v>4</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.18129496402877698</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>2.2888489208633089</v>
+        <v>2.5607913669064741</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>2.8138489208633088</v>
+        <v>3.085791366906474</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44028,11 +44028,11 @@
         <v>3</v>
       </c>
       <c r="E29" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F29" s="23">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>0.39836065573770491</v>
       </c>
       <c r="K29" s="61" t="s">
         <v>33</v>
@@ -44104,11 +44104,11 @@
         <v>1</v>
       </c>
       <c r="E32" s="53">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F32" s="23">
         <f ca="1">E32/4 * C32</f>
-        <v>0</v>
+        <v>6.6393442622950827E-2</v>
       </c>
       <c r="K32" s="21" t="s">
         <v>222</v>
@@ -44138,11 +44138,11 @@
         <v>4</v>
       </c>
       <c r="E33" s="53">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F33" s="23">
         <f ca="1">E33/4 * C33</f>
-        <v>0</v>
+        <v>0.26557377049180331</v>
       </c>
       <c r="K33" s="67" t="s">
         <v>76</v>
@@ -44174,11 +44174,11 @@
         <v>4</v>
       </c>
       <c r="E34" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F34" s="23">
         <f ca="1">E34/4 * C34</f>
-        <v>0</v>
+        <v>0.53114754098360661</v>
       </c>
       <c r="K34" s="67" t="s">
         <v>77</v>
@@ -44396,7 +44396,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>3.7844262295081976</v>
+        <v>5.0459016393442635</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44536,7 +44536,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>4.6844262295081975</v>
+        <v>5.9459016393442639</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44550,7 +44550,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>5.5488012295081974</v>
+        <v>6.8102766393442637</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: send image, typing status
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DE47A6-9201-46DA-A0A7-CD576A68D1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9B2434-2B17-4CE3-98DC-277125692B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="9" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="10" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>48.935046452480883</v>
+        <v>49.614902567588793</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44082733812949632</v>
+        <v>0.53794964028776959</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>3.085791366906474</v>
+        <v>3.7656474820143875</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>48.935046452480883</v>
+        <v>49.614902567588793</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.48935046452480885</v>
+        <v>0.49614902567588792</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>48.935046452480883</v>
+        <v>49.614902567588793</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -25086,11 +25086,11 @@
         <v>5</v>
       </c>
       <c r="E24" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F24" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.2266187050359712</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -25240,11 +25240,11 @@
         <v>10</v>
       </c>
       <c r="E31" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F31" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.4532374100719424</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>2.5607913669064741</v>
+        <v>3.2406474820143876</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>3.085791366906474</v>
+        <v>3.7656474820143875</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: get friends, debounce, infinite scroll, loading skeleton in message list
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9B2434-2B17-4CE3-98DC-277125692B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A0E8F4-9906-4E61-A18B-C7FA2F24924A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="10" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="9" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>49.614902567588793</v>
+        <v>50.022816236653547</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.53794964028776959</v>
+        <v>0.59622302158273366</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>3.7656474820143875</v>
+        <v>4.1735611510791353</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>49.614902567588793</v>
+        <v>50.02281623665354</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.49614902567588792</v>
+        <v>0.50022816236653544</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>49.614902567588793</v>
+        <v>50.022816236653547</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -24956,11 +24956,11 @@
         <v>4</v>
       </c>
       <c r="E17" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13597122302158274</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -24976,11 +24976,11 @@
         <v>4</v>
       </c>
       <c r="E18" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F18" s="65">
         <f t="shared" ref="F18:F19" ca="1" si="3">E18/4*C18</f>
-        <v>0</v>
+        <v>0.13597122302158274</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -24996,11 +24996,11 @@
         <v>4</v>
       </c>
       <c r="E19" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" s="65">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>0.13597122302158274</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>3.2406474820143876</v>
+        <v>3.6485611510791354</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>3.7656474820143875</v>
+        <v>4.1735611510791353</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: specific video page, functional copy url | update: use .env for docker
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A0E8F4-9906-4E61-A18B-C7FA2F24924A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA872C3B-014A-420B-A40D-98A35C55EA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="9" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>50.022816236653547</v>
+        <v>51.043818690904395</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23212,11 +23212,11 @@
       </c>
       <c r="D16" s="41">
         <f ca="1">E16/C16</f>
-        <v>0.5173255813953489</v>
+        <v>0.5609069767441861</v>
       </c>
       <c r="E16" s="40">
         <f ca="1">General!F58</f>
-        <v>9.8291860465116283</v>
+        <v>10.657232558139535</v>
       </c>
       <c r="G16" s="98">
         <v>0</v>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.56752305327868868</v>
+        <v>0.58360271516393458</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>6.8102766393442637</v>
+        <v>7.0032325819672154</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>50.02281623665354</v>
+        <v>51.043818690904402</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.50022816236653544</v>
+        <v>0.51043818690904397</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>50.022816236653547</v>
+        <v>51.043818690904395</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -41635,11 +41635,11 @@
         <v>2</v>
       </c>
       <c r="E28" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F28" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.29604651162790696</v>
       </c>
     </row>
     <row r="29" spans="2:6">
@@ -41695,7 +41695,7 @@
       <c r="E31" s="35"/>
       <c r="F31" s="34">
         <f ca="1">SUM(F6:F30)</f>
-        <v>7.5491860465116281</v>
+        <v>7.8452325581395348</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15.75" thickTop="1"/>
@@ -41761,11 +41761,11 @@
         <v>1</v>
       </c>
       <c r="E36" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F36" s="25">
         <f t="shared" ref="F36" ca="1" si="6">E36/4 * C36</f>
-        <v>0</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="37" spans="2:6">
@@ -41935,7 +41935,7 @@
       <c r="E45" s="35"/>
       <c r="F45" s="34">
         <f ca="1">SUM(F35:F44)</f>
-        <v>1.1400000000000001</v>
+        <v>1.292</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="15.75" thickTop="1"/>
@@ -42077,11 +42077,11 @@
         <v>20</v>
       </c>
       <c r="E54" s="131">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F54" s="25">
         <f t="shared" ca="1" si="9"/>
-        <v>0</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="55" spans="2:6" ht="15.75" customHeight="1">
@@ -42118,7 +42118,7 @@
       <c r="E56" s="35"/>
       <c r="F56" s="34">
         <f ca="1">SUM(F49:F55)</f>
-        <v>1.1400000000000001</v>
+        <v>1.5200000000000002</v>
       </c>
     </row>
     <row r="57" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -42131,7 +42131,7 @@
       <c r="E58" s="221"/>
       <c r="F58" s="107">
         <f ca="1">SUM(F31,F45,F56)</f>
-        <v>9.8291860465116283</v>
+        <v>10.657232558139535</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -43753,11 +43753,11 @@
         <v>3</v>
       </c>
       <c r="N21" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O21" s="120">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.12656250000000002</v>
       </c>
     </row>
     <row r="22" spans="2:18" ht="15.75" customHeight="1">
@@ -44048,7 +44048,7 @@
       <c r="N29" s="82"/>
       <c r="O29" s="69">
         <f ca="1">SUM(O9:O28)</f>
-        <v>0.71437499999999998</v>
+        <v>0.8409375</v>
       </c>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" thickTop="1">
@@ -44104,11 +44104,11 @@
         <v>1</v>
       </c>
       <c r="E32" s="53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F32" s="23">
         <f ca="1">E32/4 * C32</f>
-        <v>6.6393442622950827E-2</v>
+        <v>0.13278688524590165</v>
       </c>
       <c r="K32" s="21" t="s">
         <v>222</v>
@@ -44340,7 +44340,7 @@
       <c r="N39" s="237"/>
       <c r="O39" s="115">
         <f ca="1">SUM(O29,O37)</f>
-        <v>0.864375</v>
+        <v>0.99093750000000003</v>
       </c>
     </row>
     <row r="40" spans="2:15" ht="15.75" customHeight="1" thickTop="1">
@@ -44396,7 +44396,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>5.0459016393442635</v>
+        <v>5.1122950819672148</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44536,7 +44536,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>5.9459016393442639</v>
+        <v>6.0122950819672152</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44550,7 +44550,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>6.8102766393442637</v>
+        <v>7.0032325819672154</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>

</xml_diff>

<commit_message>
add: backend authentication middleware, useFollowings & useFollowers hooks | update: dark-themed modern design for every page, change followers and followings modal into a single component
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA872C3B-014A-420B-A40D-98A35C55EA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D14D9FE7-770A-4884-96C9-6DD5B9E3313C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>51.043818690904395</v>
+        <v>54.297349577532309</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23212,11 +23212,11 @@
       </c>
       <c r="D16" s="41">
         <f ca="1">E16/C16</f>
-        <v>0.5609069767441861</v>
+        <v>0.7204883720930233</v>
       </c>
       <c r="E16" s="40">
         <f ca="1">General!F58</f>
-        <v>10.657232558139535</v>
+        <v>13.689279069767442</v>
       </c>
       <c r="G16" s="98">
         <v>0</v>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.58360271516393458</v>
+        <v>0.60205974641393467</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>7.0032325819672154</v>
+        <v>7.2247169569672156</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>51.043818690904402</v>
+        <v>54.297349577532309</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.51043818690904397</v>
+        <v>0.54297349577532306</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>51.043818690904395</v>
+        <v>54.297349577532309</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -41654,11 +41654,11 @@
         <v>2</v>
       </c>
       <c r="E29" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F29" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.29604651162790696</v>
       </c>
     </row>
     <row r="30" spans="2:6">
@@ -41695,7 +41695,7 @@
       <c r="E31" s="35"/>
       <c r="F31" s="34">
         <f ca="1">SUM(F6:F30)</f>
-        <v>7.8452325581395348</v>
+        <v>8.1412790697674424</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15.75" thickTop="1"/>
@@ -41818,11 +41818,11 @@
         <v>1</v>
       </c>
       <c r="E39" s="131">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F39" s="25">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>7.5999999999999998E-2</v>
       </c>
     </row>
     <row r="40" spans="2:6">
@@ -41935,7 +41935,7 @@
       <c r="E45" s="35"/>
       <c r="F45" s="34">
         <f ca="1">SUM(F35:F44)</f>
-        <v>1.292</v>
+        <v>1.3679999999999999</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="15.75" thickTop="1"/>
@@ -42001,11 +42001,11 @@
         <v>40</v>
       </c>
       <c r="E50" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F50" s="25">
         <f t="shared" ca="1" si="9"/>
-        <v>0</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="51" spans="2:6">
@@ -42020,11 +42020,11 @@
         <v>30</v>
       </c>
       <c r="E51" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F51" s="25">
         <f t="shared" ca="1" si="9"/>
-        <v>0</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="52" spans="2:6">
@@ -42118,7 +42118,7 @@
       <c r="E56" s="35"/>
       <c r="F56" s="34">
         <f ca="1">SUM(F49:F55)</f>
-        <v>1.5200000000000002</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="57" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -42131,7 +42131,7 @@
       <c r="E58" s="221"/>
       <c r="F58" s="107">
         <f ca="1">SUM(F31,F45,F56)</f>
-        <v>10.657232558139535</v>
+        <v>13.689279069767442</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -43779,11 +43779,11 @@
         <v>3</v>
       </c>
       <c r="N22" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O22" s="120">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.12656250000000002</v>
       </c>
     </row>
     <row r="23" spans="2:18" ht="15.75" customHeight="1">
@@ -43858,11 +43858,11 @@
         <v>3</v>
       </c>
       <c r="N24" s="53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O24" s="120">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.4921875000000017E-2</v>
       </c>
     </row>
     <row r="25" spans="2:18" ht="15.75" customHeight="1">
@@ -44048,7 +44048,7 @@
       <c r="N29" s="82"/>
       <c r="O29" s="69">
         <f ca="1">SUM(O9:O28)</f>
-        <v>0.8409375</v>
+        <v>1.0624218750000001</v>
       </c>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" thickTop="1">
@@ -44340,7 +44340,7 @@
       <c r="N39" s="237"/>
       <c r="O39" s="115">
         <f ca="1">SUM(O29,O37)</f>
-        <v>0.99093750000000003</v>
+        <v>1.212421875</v>
       </c>
     </row>
     <row r="40" spans="2:15" ht="15.75" customHeight="1" thickTop="1">
@@ -44550,7 +44550,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>7.0032325819672154</v>
+        <v>7.2247169569672156</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>

</xml_diff>

<commit_message>
add: eslint & biome | update: frontend/src/* format
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D14D9FE7-770A-4884-96C9-6DD5B9E3313C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D03265-4776-4286-9366-5975818B31DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>54.297349577532309</v>
+        <v>55.185489112416029</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23212,11 +23212,11 @@
       </c>
       <c r="D16" s="41">
         <f ca="1">E16/C16</f>
-        <v>0.7204883720930233</v>
+        <v>0.76723255813953484</v>
       </c>
       <c r="E16" s="40">
         <f ca="1">General!F58</f>
-        <v>13.689279069767442</v>
+        <v>14.577418604651163</v>
       </c>
       <c r="G16" s="98">
         <v>0</v>
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>54.297349577532309</v>
+        <v>55.185489112416029</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.54297349577532306</v>
+        <v>0.55185489112416031</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>54.297349577532309</v>
+        <v>55.185489112416029</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -41540,11 +41540,11 @@
         <v>6</v>
       </c>
       <c r="E23" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F23" s="25">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.88813953488372088</v>
       </c>
     </row>
     <row r="24" spans="2:6">
@@ -41695,7 +41695,7 @@
       <c r="E31" s="35"/>
       <c r="F31" s="34">
         <f ca="1">SUM(F6:F30)</f>
-        <v>8.1412790697674424</v>
+        <v>9.0294186046511626</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15.75" thickTop="1"/>
@@ -42131,7 +42131,7 @@
       <c r="E58" s="221"/>
       <c r="F58" s="107">
         <f ca="1">SUM(F31,F45,F56)</f>
-        <v>13.689279069767442</v>
+        <v>14.577418604651163</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: rich text processor, manage videos page
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D03265-4776-4286-9366-5975818B31DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE626A3-933C-443B-B2C9-6EA1A703779A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>55.185489112416029</v>
+        <v>56.890299570416744</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -15983,8 +15983,8 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -16060,11 +16060,11 @@
         <v>1</v>
       </c>
       <c r="E4" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" s="65">
         <f ca="1">E4/4*C4</f>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -16080,11 +16080,11 @@
         <v>1</v>
       </c>
       <c r="E5" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F5" s="65">
         <f t="shared" ref="F5:F9" ca="1" si="1">E5/4*C5</f>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -16100,11 +16100,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -16120,11 +16120,11 @@
         <v>1</v>
       </c>
       <c r="E7" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -16160,11 +16160,11 @@
         <v>1</v>
       </c>
       <c r="E9" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" thickBot="1">
@@ -16183,7 +16183,7 @@
       <c r="E10" s="82"/>
       <c r="F10" s="69">
         <f ca="1">SUM(F4:F9)</f>
-        <v>0</v>
+        <v>0.83333333333333326</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" thickTop="1">
@@ -17326,11 +17326,11 @@
         <v>10</v>
       </c>
       <c r="E8" s="121">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ref="F8:F17" ca="1" si="2">E8/4*C8</f>
-        <v>0.62068965517241381</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -17346,11 +17346,11 @@
         <v>10</v>
       </c>
       <c r="E9" s="121">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0.62068965517241381</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -17366,11 +17366,11 @@
         <v>10</v>
       </c>
       <c r="E10" s="121">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0.62068965517241381</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -17386,11 +17386,11 @@
         <v>4</v>
       </c>
       <c r="E11" s="121">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.12413793103448276</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -17406,11 +17406,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="121">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.24827586206896551</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -17529,7 +17529,7 @@
       <c r="E18" s="82"/>
       <c r="F18" s="83">
         <f ca="1">SUM(F6:F15)</f>
-        <v>2.1103448275862067</v>
+        <v>0.62068965517241381</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" thickTop="1">
@@ -17582,11 +17582,11 @@
         <v>15</v>
       </c>
       <c r="E22" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" s="25">
         <f ca="1">E22/4 * C22</f>
-        <v>2.5000000000000001E-2</v>
+        <v>3.7500000000000006E-2</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -17602,11 +17602,11 @@
         <v>30</v>
       </c>
       <c r="E23" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" s="25">
         <f ca="1">E23/4 * C23</f>
-        <v>0.05</v>
+        <v>7.5000000000000011E-2</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -17622,11 +17622,11 @@
         <v>15</v>
       </c>
       <c r="E24" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" s="25">
         <f ca="1">E24/4 * C24</f>
-        <v>2.5000000000000001E-2</v>
+        <v>3.7500000000000006E-2</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -17642,11 +17642,11 @@
         <v>30</v>
       </c>
       <c r="E25" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" s="25">
         <f ca="1">E25/4 * C25</f>
-        <v>0.05</v>
+        <v>7.5000000000000011E-2</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
@@ -17662,11 +17662,11 @@
         <v>30</v>
       </c>
       <c r="E26" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" s="25">
         <f ca="1">E26/4 * C26</f>
-        <v>0.05</v>
+        <v>7.5000000000000011E-2</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
@@ -17684,7 +17684,7 @@
       <c r="E27" s="35"/>
       <c r="F27" s="34">
         <f ca="1">SUM(F22:F26)</f>
-        <v>0.2</v>
+        <v>0.30000000000000004</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -17697,7 +17697,7 @@
       <c r="E29" s="238"/>
       <c r="F29" s="107">
         <f ca="1">SUM(,F18,F27)</f>
-        <v>2.3103448275862069</v>
+        <v>0.92068965517241386</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -20031,11 +20031,11 @@
         <v>2</v>
       </c>
       <c r="E11" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -20071,11 +20071,11 @@
         <v>5</v>
       </c>
       <c r="E13" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F13" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.3125</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -20091,11 +20091,11 @@
         <v>3</v>
       </c>
       <c r="E14" s="122">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>4.6875E-2</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -20214,7 +20214,7 @@
       <c r="E20" s="82"/>
       <c r="F20" s="83">
         <f ca="1">SUM(F6:F19)</f>
-        <v>2.25</v>
+        <v>2.734375</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" thickTop="1">
@@ -20389,7 +20389,7 @@
       <c r="E31" s="238"/>
       <c r="F31" s="107">
         <f ca="1">SUM(F20,F29)</f>
-        <v>2.625</v>
+        <v>3.109375</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" thickTop="1">
@@ -21487,11 +21487,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="65">
         <f ca="1">E6/4*C6</f>
-        <v>0</v>
+        <v>4.3902439024390248E-2</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -21507,11 +21507,11 @@
         <v>1</v>
       </c>
       <c r="E7" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f ca="1">E7/4*C7</f>
-        <v>0</v>
+        <v>4.3902439024390248E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -21527,11 +21527,11 @@
         <v>3</v>
       </c>
       <c r="E8" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ref="F8:F25" ca="1" si="1">E8/4*C8</f>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
       <c r="H8" s="134" t="s">
         <v>322</v>
@@ -21554,14 +21554,14 @@
       </c>
       <c r="E9" s="4">
         <f>H9/I9*4</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.16463414634146342</v>
       </c>
       <c r="H9" s="138">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I9" s="136">
         <v>12</v>
@@ -21667,11 +21667,11 @@
         <v>6</v>
       </c>
       <c r="E14" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.26341463414634148</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -21707,11 +21707,11 @@
         <v>3</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -21727,11 +21727,11 @@
         <v>3</v>
       </c>
       <c r="E17" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -21787,11 +21787,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F20" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -21807,11 +21807,11 @@
         <v>3</v>
       </c>
       <c r="E21" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F21" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -21827,11 +21827,11 @@
         <v>2</v>
       </c>
       <c r="E22" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F22" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>8.7804878048780496E-2</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -21847,11 +21847,11 @@
         <v>6</v>
       </c>
       <c r="E23" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F23" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.26341463414634148</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -21910,7 +21910,7 @@
       <c r="E26" s="82"/>
       <c r="F26" s="83">
         <f ca="1">SUM(F6:F25)</f>
-        <v>0</v>
+        <v>1.525609756097561</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" thickTop="1">
@@ -21963,11 +21963,11 @@
         <v>15</v>
       </c>
       <c r="E30" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F30" s="25">
         <f ca="1">E30/4 * C30</f>
-        <v>0</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -21983,11 +21983,11 @@
         <v>10</v>
       </c>
       <c r="E31" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F31" s="25">
         <f ca="1">E31/4 * C31</f>
-        <v>0</v>
+        <v>3.0000000000000006E-2</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -22003,11 +22003,11 @@
         <v>15</v>
       </c>
       <c r="E32" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F32" s="25">
         <f ca="1">E32/4 * C32</f>
-        <v>0</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -22023,11 +22023,11 @@
         <v>30</v>
       </c>
       <c r="E33" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F33" s="25">
         <f ca="1">E33/4 * C33</f>
-        <v>0</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1">
@@ -22043,11 +22043,11 @@
         <v>30</v>
       </c>
       <c r="E34" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" s="25">
         <f ca="1">E34/4 * C34</f>
-        <v>0</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" thickBot="1">
@@ -22065,7 +22065,7 @@
       <c r="E35" s="35"/>
       <c r="F35" s="34">
         <f ca="1">SUM(F30:F34)</f>
-        <v>0</v>
+        <v>0.30000000000000004</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -22078,7 +22078,7 @@
       <c r="E37" s="238"/>
       <c r="F37" s="107">
         <f ca="1">SUM(,F26,F35)</f>
-        <v>0</v>
+        <v>1.825609756097561</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.60205974641393467</v>
+        <v>0.64632204149590178</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>7.2247169569672156</v>
+        <v>7.7558644979508209</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23418,11 +23418,11 @@
       </c>
       <c r="D27" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.83333333333333326</v>
       </c>
       <c r="E27" s="40">
         <f ca="1">'Rich Text'!F10</f>
-        <v>0</v>
+        <v>0.83333333333333326</v>
       </c>
     </row>
     <row r="28" spans="2:8">
@@ -23434,11 +23434,11 @@
       </c>
       <c r="D28" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.57758620689655171</v>
+        <v>0.23017241379310346</v>
       </c>
       <c r="E28" s="40">
         <f ca="1">'Settings Page'!F29</f>
-        <v>2.3103448275862069</v>
+        <v>0.92068965517241386</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23466,11 +23466,11 @@
       </c>
       <c r="D30" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.62187499999999996</v>
       </c>
       <c r="E30" s="40">
         <f ca="1">'Studio Upload Page'!F31</f>
-        <v>2.625</v>
+        <v>3.109375</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -23482,11 +23482,11 @@
       </c>
       <c r="D31" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.45640243902439026</v>
       </c>
       <c r="E31" s="40">
         <f ca="1">'Studio Post Page'!F37</f>
-        <v>0</v>
+        <v>1.825609756097561</v>
       </c>
     </row>
     <row r="32" spans="2:8">
@@ -23531,11 +23531,11 @@
       </c>
       <c r="D34" s="41">
         <f ca="1">E34/C34</f>
-        <v>0.67000000000000015</v>
+        <v>0.59750000000000014</v>
       </c>
       <c r="E34" s="40" cm="1">
         <f t="array" aca="1" ref="E34" ca="1">INDIRECT("'" &amp; $D$8 &amp; "'!A1")</f>
-        <v>5.3600000000000012</v>
+        <v>4.7800000000000011</v>
       </c>
       <c r="K34" s="43"/>
     </row>
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>55.185489112416029</v>
+        <v>56.890299570416744</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.55185489112416031</v>
+        <v>0.56890299570416747</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>55.185489112416029</v>
+        <v>56.890299570416744</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -33241,7 +33241,7 @@
     <row r="1" spans="1:6" ht="15" customHeight="1">
       <c r="A1" s="110">
         <f ca="1">F13</f>
-        <v>5.3600000000000012</v>
+        <v>4.7800000000000011</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -33286,11 +33286,11 @@
         <v>8</v>
       </c>
       <c r="E4" s="121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="65">
         <f ca="1">E4/4*C4</f>
-        <v>0.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
@@ -33324,11 +33324,11 @@
         <v>15</v>
       </c>
       <c r="E6" s="121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -33381,11 +33381,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -33460,7 +33460,7 @@
       <c r="E13" s="84"/>
       <c r="F13" s="83">
         <f ca="1">SUM(F4:F12)</f>
-        <v>5.3600000000000012</v>
+        <v>4.7800000000000011</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickTop="1"/>
@@ -43520,11 +43520,11 @@
         <v>2</v>
       </c>
       <c r="E15" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>0.26557377049180331</v>
       </c>
       <c r="K15" s="118" t="s">
         <v>250</v>
@@ -43841,11 +43841,11 @@
         <v>2</v>
       </c>
       <c r="E24" s="53">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F24" s="23">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>0.26557377049180331</v>
       </c>
       <c r="K24" s="118" t="s">
         <v>72</v>
@@ -44396,7 +44396,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>5.1122950819672148</v>
+        <v>5.6434426229508201</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44536,7 +44536,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>6.0122950819672152</v>
+        <v>6.5434426229508205</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44550,7 +44550,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>7.2247169569672156</v>
+        <v>7.7558644979508209</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: edit video page | update: manage videos, isPublished in Video model for draft
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE626A3-933C-443B-B2C9-6EA1A703779A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FC517E-3E6F-48C2-B578-83A80E4E1024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>56.890299570416744</v>
+        <v>58.112708107002106</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -20131,11 +20131,11 @@
         <v>5</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.15625</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -20151,11 +20151,11 @@
         <v>5</v>
       </c>
       <c r="E17" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.3125</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -20214,7 +20214,7 @@
       <c r="E20" s="82"/>
       <c r="F20" s="83">
         <f ca="1">SUM(F6:F19)</f>
-        <v>2.734375</v>
+        <v>3.203125</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" thickTop="1">
@@ -20389,7 +20389,7 @@
       <c r="E31" s="238"/>
       <c r="F31" s="107">
         <f ca="1">SUM(F20,F29)</f>
-        <v>3.109375</v>
+        <v>3.578125</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" thickTop="1">
@@ -21580,11 +21580,11 @@
         <v>3</v>
       </c>
       <c r="E10" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -21601,14 +21601,14 @@
       </c>
       <c r="E11" s="4">
         <f>H11/I11*4</f>
-        <v>0</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.18292682926829268</v>
       </c>
       <c r="H11" s="138">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I11" s="136">
         <v>6</v>
@@ -21627,11 +21627,11 @@
         <v>10</v>
       </c>
       <c r="E12" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.21951219512195122</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -21647,11 +21647,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.21951219512195122</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -21667,11 +21667,11 @@
         <v>6</v>
       </c>
       <c r="E14" s="122">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0.26341463414634148</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -21687,11 +21687,11 @@
         <v>6</v>
       </c>
       <c r="E15" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F15" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.13170731707317074</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -21910,7 +21910,7 @@
       <c r="E26" s="82"/>
       <c r="F26" s="83">
         <f ca="1">SUM(F6:F25)</f>
-        <v>1.525609756097561</v>
+        <v>2.2792682926829277</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" thickTop="1">
@@ -22078,7 +22078,7 @@
       <c r="E37" s="238"/>
       <c r="F37" s="107">
         <f ca="1">SUM(,F26,F35)</f>
-        <v>1.825609756097561</v>
+        <v>2.5792682926829276</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23466,11 +23466,11 @@
       </c>
       <c r="D30" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.62187499999999996</v>
+        <v>0.71562499999999996</v>
       </c>
       <c r="E30" s="40">
         <f ca="1">'Studio Upload Page'!F31</f>
-        <v>3.109375</v>
+        <v>3.578125</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -23482,11 +23482,11 @@
       </c>
       <c r="D31" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.45640243902439026</v>
+        <v>0.64481707317073189</v>
       </c>
       <c r="E31" s="40">
         <f ca="1">'Studio Post Page'!F37</f>
-        <v>1.825609756097561</v>
+        <v>2.5792682926829276</v>
       </c>
     </row>
     <row r="32" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>56.890299570416744</v>
+        <v>58.112708107002106</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.56890299570416747</v>
+        <v>0.58112708107002109</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>56.890299570416744</v>
+        <v>58.112708107002106</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: hot reload for auth-service
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FC517E-3E6F-48C2-B578-83A80E4E1024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DE1459-8677-48BC-A2E0-0E11E20A1F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>58.112708107002106</v>
+        <v>58.525637735513122</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11364,11 +11364,11 @@
         <v>1</v>
       </c>
       <c r="E17" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2.3376623376623377E-2</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -11739,11 +11739,11 @@
         <v>4</v>
       </c>
       <c r="E34" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34" s="163">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.350649350649351E-2</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -11842,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>1.8567717996289428</v>
+        <v>1.9736549165120596</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -12001,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>2.2567717996289427</v>
+        <v>2.3736549165120597</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23212,11 +23212,11 @@
       </c>
       <c r="D16" s="41">
         <f ca="1">E16/C16</f>
-        <v>0.76723255813953484</v>
+        <v>0.78281395348837213</v>
       </c>
       <c r="E16" s="40">
         <f ca="1">General!F58</f>
-        <v>14.577418604651163</v>
+        <v>14.873465116279069</v>
       </c>
       <c r="G16" s="98">
         <v>0</v>
@@ -23370,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.56419294990723567</v>
+        <v>0.59341372912801493</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>2.2567717996289427</v>
+        <v>2.3736549165120597</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>58.112708107002106</v>
+        <v>58.525637735513129</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.58112708107002109</v>
+        <v>0.58525637735513125</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>58.112708107002106</v>
+        <v>58.525637735513122</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -41559,11 +41559,11 @@
         <v>2</v>
       </c>
       <c r="E24" s="131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F24" s="25">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.29604651162790696</v>
       </c>
     </row>
     <row r="25" spans="2:6">
@@ -41695,7 +41695,7 @@
       <c r="E31" s="35"/>
       <c r="F31" s="34">
         <f ca="1">SUM(F6:F30)</f>
-        <v>9.0294186046511626</v>
+        <v>9.3254651162790694</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15.75" thickTop="1"/>
@@ -42131,7 +42131,7 @@
       <c r="E58" s="221"/>
       <c r="F58" s="107">
         <f ca="1">SUM(F31,F45,F56)</f>
-        <v>14.577418604651163</v>
+        <v>14.873465116279069</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: caption generator with timestamps, live streamer & viewer page, hot reload for user-service
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DE1459-8677-48BC-A2E0-0E11E20A1F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7367CF65-79E7-439E-88ED-EFF2461BB320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>58.525637735513122</v>
+        <v>61.675258139605496</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11404,11 +11404,11 @@
         <v>3</v>
       </c>
       <c r="E19" s="122">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F19" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0.14025974025974025</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -11652,11 +11652,11 @@
         <v>2</v>
       </c>
       <c r="E30" s="122">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F30" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>9.350649350649351E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -11842,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>1.9736549165120596</v>
+        <v>1.7398886827458258</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -12001,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>2.3736549165120597</v>
+        <v>2.1398886827458257</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13220,11 +13220,11 @@
         <v>2</v>
       </c>
       <c r="E13" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F13" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -13303,7 +13303,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>1.605</v>
+        <v>1.7250000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13452,7 +13452,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>1.7549999999999999</v>
+        <v>1.875</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -17446,11 +17446,11 @@
         <v>6</v>
       </c>
       <c r="E14" s="121">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.3724137931034483</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -17529,7 +17529,7 @@
       <c r="E18" s="82"/>
       <c r="F18" s="83">
         <f ca="1">SUM(F6:F15)</f>
-        <v>0.62068965517241381</v>
+        <v>0.99310344827586217</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" thickTop="1">
@@ -17697,7 +17697,7 @@
       <c r="E29" s="238"/>
       <c r="F29" s="107">
         <f ca="1">SUM(,F18,F27)</f>
-        <v>0.92068965517241386</v>
+        <v>1.2931034482758621</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23278,11 +23278,11 @@
       </c>
       <c r="D19" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.66250000000000009</v>
+        <v>0.69464285714285723</v>
       </c>
       <c r="E19" s="40">
         <f ca="1">'Sign Up Page'!F34</f>
-        <v>1.9875000000000003</v>
+        <v>2.0839285714285718</v>
       </c>
       <c r="G19" s="42">
         <v>3</v>
@@ -23370,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.59341372912801493</v>
+        <v>0.53497217068645642</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>2.3736549165120597</v>
+        <v>2.1398886827458257</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23386,11 +23386,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.87749999999999995</v>
+        <v>0.9375</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>1.7549999999999999</v>
+        <v>1.875</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23434,11 +23434,11 @@
       </c>
       <c r="D28" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.23017241379310346</v>
+        <v>0.32327586206896552</v>
       </c>
       <c r="E28" s="40">
         <f ca="1">'Settings Page'!F29</f>
-        <v>0.92068965517241386</v>
+        <v>1.2931034482758621</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.59622302158273366</v>
+        <v>0.60269784172661856</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>4.1735611510791353</v>
+        <v>4.2188848920863302</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23514,11 +23514,11 @@
       </c>
       <c r="D33" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>8.1844106463878324E-2</v>
       </c>
       <c r="E33" s="40">
         <f ca="1">Live!F47</f>
-        <v>0</v>
+        <v>0.40922053231939165</v>
       </c>
     </row>
     <row r="34" spans="2:16">
@@ -23531,11 +23531,11 @@
       </c>
       <c r="D34" s="41">
         <f ca="1">E34/C34</f>
-        <v>0.59750000000000014</v>
+        <v>0.89000000000000012</v>
       </c>
       <c r="E34" s="40" cm="1">
         <f t="array" aca="1" ref="E34" ca="1">INDIRECT("'" &amp; $D$8 &amp; "'!A1")</f>
-        <v>4.7800000000000011</v>
+        <v>7.120000000000001</v>
       </c>
       <c r="K34" s="43"/>
     </row>
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>58.525637735513129</v>
+        <v>61.675258139605496</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.58525637735513125</v>
+        <v>0.61675258139605493</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>58.525637735513122</v>
+        <v>61.675258139605496</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -25194,14 +25194,14 @@
       </c>
       <c r="E29" s="4">
         <f>H29/I29*4</f>
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="F29" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>4.5323741007194246E-2</v>
+        <v>9.0647482014388492E-2</v>
       </c>
       <c r="H29" s="135">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29" s="136">
         <v>5</v>
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>3.6485611510791354</v>
+        <v>3.6938848920863299</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>4.1735611510791353</v>
+        <v>4.2188848920863302</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -26568,11 +26568,11 @@
         <v>1</v>
       </c>
       <c r="E7" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" s="65">
         <f ca="1">E7/4*C7</f>
-        <v>0</v>
+        <v>1.7110266159695818E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -26588,11 +26588,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ref="F8:F36" ca="1" si="0">E8/4*C8</f>
-        <v>0</v>
+        <v>1.7110266159695818E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -27181,7 +27181,7 @@
       <c r="E37" s="82"/>
       <c r="F37" s="83">
         <f ca="1">SUM(F7:F36)</f>
-        <v>0</v>
+        <v>3.4220532319391636E-2</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" thickTop="1">
@@ -27234,11 +27234,11 @@
         <v>15</v>
       </c>
       <c r="E41" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F41" s="25">
         <f ca="1">E41/4 * C41</f>
-        <v>0</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="15.75" customHeight="1">
@@ -27254,11 +27254,11 @@
         <v>15</v>
       </c>
       <c r="E42" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F42" s="25">
         <f ca="1">E42/4 * C42</f>
-        <v>0</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" customHeight="1">
@@ -27273,11 +27273,11 @@
         <v>30</v>
       </c>
       <c r="E43" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F43" s="25">
         <f ca="1">E43/4 * C43</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="15.75" customHeight="1">
@@ -27292,11 +27292,11 @@
         <v>30</v>
       </c>
       <c r="E44" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F44" s="25">
         <f ca="1">E44/4 * C44</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" thickBot="1">
@@ -27314,7 +27314,7 @@
       <c r="E45" s="35"/>
       <c r="F45" s="34">
         <f ca="1">SUM(F41:F44)</f>
-        <v>0</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" thickTop="1"/>
@@ -27327,7 +27327,7 @@
       <c r="E47" s="238"/>
       <c r="F47" s="107">
         <f ca="1">SUM(F37,F45)</f>
-        <v>0</v>
+        <v>0.40922053231939165</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" thickTop="1"/>
@@ -33241,7 +33241,7 @@
     <row r="1" spans="1:6" ht="15" customHeight="1">
       <c r="A1" s="110">
         <f ca="1">F13</f>
-        <v>4.7800000000000011</v>
+        <v>7.120000000000001</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -33286,11 +33286,11 @@
         <v>8</v>
       </c>
       <c r="E4" s="121">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" s="65">
         <f ca="1">E4/4*C4</f>
-        <v>0</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
@@ -33305,11 +33305,11 @@
         <v>15</v>
       </c>
       <c r="E5" s="121">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" s="65">
         <f t="shared" ref="F5:F11" ca="1" si="1">E5/4*C5</f>
-        <v>0.3</v>
+        <v>0.89999999999999991</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -33324,11 +33324,11 @@
         <v>15</v>
       </c>
       <c r="E6" s="121">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F6" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.89999999999999991</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -33381,11 +33381,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="121">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -33460,7 +33460,7 @@
       <c r="E13" s="84"/>
       <c r="F13" s="83">
         <f ca="1">SUM(F4:F12)</f>
-        <v>4.7800000000000011</v>
+        <v>7.120000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" thickTop="1"/>
@@ -45929,11 +45929,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F20" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>9.6428571428571433E-2</v>
       </c>
     </row>
     <row r="21" spans="2:6">
@@ -45989,7 +45989,7 @@
       <c r="E23" s="52"/>
       <c r="F23" s="62">
         <f ca="1">SUM(F6:F22)</f>
-        <v>1.6875000000000002</v>
+        <v>1.7839285714285718</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="15.75" thickTop="1"/>
@@ -46148,7 +46148,7 @@
       <c r="E34" s="238"/>
       <c r="F34" s="107">
         <f ca="1">SUM(F23,F32)</f>
-        <v>1.9875000000000003</v>
+        <v>2.0839285714285718</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: advertisement, hot reload for video-service
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7367CF65-79E7-439E-88ED-EFF2461BB320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A281E5B1-9C48-4258-ABBD-8DAFCF3C4B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>61.675258139605496</v>
+        <v>62.675258139605496</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -18767,11 +18767,11 @@
         <v>4</v>
       </c>
       <c r="E4" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" s="65">
         <f ca="1">E4/4*C4</f>
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -18787,11 +18787,11 @@
         <v>10</v>
       </c>
       <c r="E5" s="122">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F5" s="65">
         <f t="shared" ref="F5" ca="1" si="0">E5/4*C5</f>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75" thickBot="1">
@@ -18810,7 +18810,7 @@
       <c r="E6" s="82"/>
       <c r="F6" s="69">
         <f ca="1">SUM(F4:F5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickTop="1">
@@ -23450,11 +23450,11 @@
       </c>
       <c r="D29" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="40">
         <f ca="1">Advertisement!F6</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>61.675258139605496</v>
+        <v>62.675258139605496</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.61675258139605493</v>
+        <v>0.62675258139605494</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>61.675258139605496</v>
+        <v>62.675258139605496</v>
       </c>
       <c r="E41" s="203"/>
     </row>

</xml_diff>

<commit_message>
add: live stream (camera, screen, audio)
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A281E5B1-9C48-4258-ABBD-8DAFCF3C4B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B771DF2F-CCE7-42A2-AB80-8D9AF3B4B4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>62.675258139605496</v>
+        <v>64.507767645308917</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23514,11 +23514,11 @@
       </c>
       <c r="D33" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>8.1844106463878324E-2</v>
+        <v>0.44834600760456278</v>
       </c>
       <c r="E33" s="40">
         <f ca="1">Live!F47</f>
-        <v>0.40922053231939165</v>
+        <v>2.2417300380228138</v>
       </c>
     </row>
     <row r="34" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>62.675258139605496</v>
+        <v>64.507767645308917</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.62675258139605494</v>
+        <v>0.64507767645308922</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>62.675258139605496</v>
+        <v>64.507767645308917</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -26712,14 +26712,14 @@
       </c>
       <c r="E14" s="4">
         <f>H14/I14*4</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>2.7376425855513309E-2</v>
       </c>
       <c r="H14" s="138">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="136">
         <v>5</v>
@@ -26758,11 +26758,11 @@
         <v>12</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.10266159695817491</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -26778,11 +26778,11 @@
         <v>4</v>
       </c>
       <c r="E17" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3.4220532319391636E-2</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -26818,11 +26818,11 @@
         <v>30</v>
       </c>
       <c r="E19" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.38498098859315594</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -26838,11 +26838,11 @@
         <v>30</v>
       </c>
       <c r="E20" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.38498098859315594</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -26858,14 +26858,14 @@
         <v>20</v>
       </c>
       <c r="E21" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.25665399239543724</v>
       </c>
       <c r="H21" s="138">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I21" s="136">
         <v>8</v>
@@ -26885,11 +26885,11 @@
       </c>
       <c r="E22" s="4">
         <f>H21/I21*4</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1.7110266159695818E-2</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -26905,11 +26905,11 @@
         <v>8</v>
       </c>
       <c r="E23" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.10266159695817491</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -26925,11 +26925,11 @@
         <v>15</v>
       </c>
       <c r="E24" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.12832699619771865</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -26945,11 +26945,11 @@
         <v>4</v>
       </c>
       <c r="E25" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F25" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3.4220532319391636E-2</v>
       </c>
       <c r="H25" s="100"/>
     </row>
@@ -26996,11 +26996,11 @@
         <v>5</v>
       </c>
       <c r="E28" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F28" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>6.4163498098859309E-2</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -27057,11 +27057,11 @@
         <v>12</v>
       </c>
       <c r="E31" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F31" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.10266159695817491</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -27097,11 +27097,11 @@
         <v>15</v>
       </c>
       <c r="E33" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F33" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.19249049429657797</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -27181,7 +27181,7 @@
       <c r="E37" s="82"/>
       <c r="F37" s="83">
         <f ca="1">SUM(F7:F36)</f>
-        <v>3.4220532319391636E-2</v>
+        <v>1.8667300380228138</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" thickTop="1">
@@ -27327,7 +27327,7 @@
       <c r="E47" s="238"/>
       <c r="F47" s="107">
         <f ca="1">SUM(F37,F45)</f>
-        <v>0.40922053231939165</v>
+        <v>2.2417300380228138</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,6 +51522,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51744,16 +51753,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51772,14 +51780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: toggle streamer's video
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B771DF2F-CCE7-42A2-AB80-8D9AF3B4B4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002C1C66-EA00-49EF-99B4-70992B6E3B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>64.507767645308917</v>
+        <v>64.627539508426793</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -23514,11 +23514,11 @@
       </c>
       <c r="D33" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44834600760456278</v>
+        <v>0.47230038022813686</v>
       </c>
       <c r="E33" s="40">
         <f ca="1">Live!F47</f>
-        <v>2.2417300380228138</v>
+        <v>2.3615019011406844</v>
       </c>
     </row>
     <row r="34" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>64.507767645308917</v>
+        <v>64.627539508426793</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.64507767645308922</v>
+        <v>0.6462753950842679</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>64.507767645308917</v>
+        <v>64.627539508426793</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -27037,11 +27037,11 @@
         <v>2</v>
       </c>
       <c r="E30" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F30" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1.7110266159695818E-2</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -27117,11 +27117,11 @@
         <v>8</v>
       </c>
       <c r="E34" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>0.10266159695817491</v>
       </c>
       <c r="H34" s="100"/>
     </row>
@@ -27181,7 +27181,7 @@
       <c r="E37" s="82"/>
       <c r="F37" s="83">
         <f ca="1">SUM(F7:F36)</f>
-        <v>1.8667300380228138</v>
+        <v>1.9865019011406846</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" thickTop="1">
@@ -27327,7 +27327,7 @@
       <c r="E47" s="238"/>
       <c r="F47" s="107">
         <f ca="1">SUM(F37,F45)</f>
-        <v>2.2417300380228138</v>
+        <v>2.3615019011406844</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51744,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51772,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: google login & register
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4C63213-82F7-4709-9B55-6519C070BBF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E23A43-4BD4-4C84-B816-1E21024A8E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="16" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>64.627539508426793</v>
+        <v>66.304310794810192</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11169,14 +11169,14 @@
       </c>
       <c r="E8" s="3">
         <f>H8*4/I8</f>
-        <v>3.4285714285714284</v>
+        <v>4</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0148423005565864E-2</v>
+        <v>9.350649350649351E-2</v>
       </c>
       <c r="H8" s="138">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="136">
         <v>7</v>
@@ -11282,11 +11282,11 @@
         <v>2</v>
       </c>
       <c r="E13" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>4.6753246753246755E-2</v>
+        <v>7.0129870129870125E-2</v>
       </c>
       <c r="H13" s="169"/>
       <c r="I13" s="170"/>
@@ -11842,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>1.7398886827458258</v>
+        <v>1.7766233766233768</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -12001,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>2.1398886827458257</v>
+        <v>2.1766233766233767</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -13080,11 +13080,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="65">
         <f ca="1">E6/4*C6</f>
-        <v>0.03</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -13303,7 +13303,7 @@
       <c r="E17" s="82"/>
       <c r="F17" s="69">
         <f ca="1">SUM(F6:F16)</f>
-        <v>1.7250000000000001</v>
+        <v>1.7400000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickTop="1">
@@ -13452,7 +13452,7 @@
       <c r="E27" s="238"/>
       <c r="F27" s="107">
         <f ca="1">SUM(F17,F25)</f>
-        <v>1.875</v>
+        <v>1.8900000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.64632204149590178</v>
+        <v>0.66508997182377072</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>7.7558644979508209</v>
+        <v>7.9810796618852482</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23256,11 +23256,11 @@
       </c>
       <c r="D18" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.41500000000000004</v>
+        <v>0.78250000000000008</v>
       </c>
       <c r="E18" s="40">
         <f ca="1">'Login Page'!F28</f>
-        <v>1.2450000000000001</v>
+        <v>2.3475000000000001</v>
       </c>
       <c r="G18" s="42">
         <v>2</v>
@@ -23278,11 +23278,11 @@
       </c>
       <c r="D19" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.69464285714285723</v>
+        <v>0.79375000000000018</v>
       </c>
       <c r="E19" s="40">
         <f ca="1">'Sign Up Page'!F34</f>
-        <v>2.0839285714285718</v>
+        <v>2.3812500000000005</v>
       </c>
       <c r="G19" s="42">
         <v>3</v>
@@ -23370,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.53497217068645642</v>
+        <v>0.54415584415584417</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>2.1398886827458257</v>
+        <v>2.1766233766233767</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23386,11 +23386,11 @@
       </c>
       <c r="D25" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.9375</v>
+        <v>0.94500000000000006</v>
       </c>
       <c r="E25" s="40">
         <f ca="1">'Create Playlist Page'!F27</f>
-        <v>1.875</v>
+        <v>1.8900000000000001</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>64.627539508426793</v>
+        <v>66.304310794810192</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.6462753950842679</v>
+        <v>0.66304310794810195</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>64.627539508426793</v>
+        <v>66.304310794810192</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -43350,15 +43350,14 @@
       </c>
       <c r="N10" s="54">
         <f>Q10*4/R10</f>
-        <v>1.2</v>
+        <v>3.6</v>
       </c>
       <c r="O10" s="120">
         <f t="shared" ca="1" si="1"/>
-        <v>2.5312500000000002E-2</v>
+        <v>7.5937500000000005E-2</v>
       </c>
       <c r="Q10" s="144">
-        <f>1+0+1+1+0</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="R10" s="25">
         <v>10</v>
@@ -43700,11 +43699,11 @@
         <v>1</v>
       </c>
       <c r="E20" s="53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F20" s="152">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>9.959016393442624E-2</v>
       </c>
       <c r="K20" s="118" t="s">
         <v>69</v>
@@ -44048,7 +44047,7 @@
       <c r="N29" s="82"/>
       <c r="O29" s="69">
         <f ca="1">SUM(O9:O28)</f>
-        <v>1.0624218750000001</v>
+        <v>1.1130468750000002</v>
       </c>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" thickTop="1">
@@ -44155,11 +44154,11 @@
         <v>2</v>
       </c>
       <c r="N33" s="53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O33" s="23">
         <f ca="1">N33/4 * L33</f>
-        <v>4.2857142857142864E-2</v>
+        <v>6.4285714285714293E-2</v>
       </c>
     </row>
     <row r="34" spans="2:15" ht="15.75" customHeight="1">
@@ -44191,11 +44190,11 @@
         <v>3</v>
       </c>
       <c r="N34" s="53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O34" s="23">
         <f ca="1">N34/4 * L34</f>
-        <v>6.4285714285714293E-2</v>
+        <v>9.6428571428571447E-2</v>
       </c>
     </row>
     <row r="35" spans="2:15" ht="15.75" customHeight="1">
@@ -44217,11 +44216,11 @@
         <v>1</v>
       </c>
       <c r="N35" s="53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O35" s="23">
         <f ca="1">N35/4 * L35</f>
-        <v>2.1428571428571432E-2</v>
+        <v>3.2142857142857147E-2</v>
       </c>
     </row>
     <row r="36" spans="2:15" ht="15.75" customHeight="1">
@@ -44253,11 +44252,11 @@
         <v>1</v>
       </c>
       <c r="N36" s="53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O36" s="23">
         <f ca="1">N36/4 * L36</f>
-        <v>2.1428571428571432E-2</v>
+        <v>3.2142857142857147E-2</v>
       </c>
     </row>
     <row r="37" spans="2:15" ht="15.75" customHeight="1" thickBot="1">
@@ -44292,7 +44291,7 @@
       <c r="N37" s="35"/>
       <c r="O37" s="62">
         <f ca="1">SUM(O33:O36)</f>
-        <v>0.15000000000000002</v>
+        <v>0.22500000000000003</v>
       </c>
     </row>
     <row r="38" spans="2:15" ht="15.75" customHeight="1" thickTop="1">
@@ -44340,7 +44339,7 @@
       <c r="N39" s="237"/>
       <c r="O39" s="115">
         <f ca="1">SUM(O29,O37)</f>
-        <v>1.212421875</v>
+        <v>1.3380468750000003</v>
       </c>
     </row>
     <row r="40" spans="2:15" ht="15.75" customHeight="1" thickTop="1">
@@ -44396,7 +44395,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>5.6434426229508201</v>
+        <v>5.743032786885248</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44536,7 +44535,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>6.5434426229508205</v>
+        <v>6.6430327868852483</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44550,7 +44549,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>7.7558644979508209</v>
+        <v>7.9810796618852482</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -45853,11 +45852,11 @@
         <v>20</v>
       </c>
       <c r="E16" s="122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.32142857142857145</v>
       </c>
     </row>
     <row r="17" spans="2:6">
@@ -45929,11 +45928,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="122">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>9.6428571428571433E-2</v>
+        <v>7.2321428571428578E-2</v>
       </c>
     </row>
     <row r="21" spans="2:6">
@@ -45989,7 +45988,7 @@
       <c r="E23" s="52"/>
       <c r="F23" s="62">
         <f ca="1">SUM(F6:F22)</f>
-        <v>1.7839285714285718</v>
+        <v>2.0812500000000003</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="15.75" thickTop="1"/>
@@ -46148,7 +46147,7 @@
       <c r="E34" s="238"/>
       <c r="F34" s="107">
         <f ca="1">SUM(F23,F32)</f>
-        <v>2.0839285714285718</v>
+        <v>2.3812500000000005</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -47334,11 +47333,11 @@
         <v>10</v>
       </c>
       <c r="E11" s="121">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="12" spans="2:9">
@@ -47391,11 +47390,11 @@
         <v>3</v>
       </c>
       <c r="E14" s="121">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>0.20250000000000001</v>
       </c>
     </row>
     <row r="15" spans="2:9">
@@ -47451,7 +47450,7 @@
       <c r="E17" s="52"/>
       <c r="F17" s="62">
         <f ca="1">SUM(F6:F16)</f>
-        <v>0.94500000000000006</v>
+        <v>2.0475000000000003</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="15.75" thickTop="1"/>
@@ -47610,7 +47609,7 @@
       <c r="E28" s="238"/>
       <c r="F28" s="107">
         <f ca="1">SUM(F17,F26)</f>
-        <v>1.2450000000000001</v>
+        <v>2.3475000000000001</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51522,15 +51521,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51753,15 +51743,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51780,6 +51771,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: extra  notification and content settings attribute in User model
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E23A43-4BD4-4C84-B816-1E21024A8E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006879FB-6192-4DD0-B157-6CDBD95D8106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>66.304310794810192</v>
+        <v>66.645690105155012</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -17326,11 +17326,11 @@
         <v>10</v>
       </c>
       <c r="E8" s="121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="65">
         <f t="shared" ref="F8:F17" ca="1" si="2">E8/4*C8</f>
-        <v>0</v>
+        <v>0.15517241379310345</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -17346,11 +17346,11 @@
         <v>10</v>
       </c>
       <c r="E9" s="121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.15517241379310345</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -17366,11 +17366,11 @@
         <v>10</v>
       </c>
       <c r="E10" s="121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>0.15517241379310345</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -17406,11 +17406,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0.24827586206896551</v>
+        <v>6.2068965517241378E-2</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -17426,11 +17426,11 @@
         <v>4</v>
       </c>
       <c r="E13" s="121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="65">
         <f ca="1">E13/4*C13</f>
-        <v>0</v>
+        <v>6.2068965517241378E-2</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -17529,7 +17529,7 @@
       <c r="E18" s="82"/>
       <c r="F18" s="83">
         <f ca="1">SUM(F6:F15)</f>
-        <v>0.99310344827586217</v>
+        <v>1.3344827586206895</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" thickTop="1">
@@ -17697,7 +17697,7 @@
       <c r="E29" s="238"/>
       <c r="F29" s="107">
         <f ca="1">SUM(,F18,F27)</f>
-        <v>1.2931034482758621</v>
+        <v>1.6344827586206896</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23434,11 +23434,11 @@
       </c>
       <c r="D28" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.32327586206896552</v>
+        <v>0.4086206896551724</v>
       </c>
       <c r="E28" s="40">
         <f ca="1">'Settings Page'!F29</f>
-        <v>1.2931034482758621</v>
+        <v>1.6344827586206896</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>66.304310794810192</v>
+        <v>66.645690105155012</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.66304310794810195</v>
+        <v>0.66645690105155009</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>66.304310794810192</v>
+        <v>66.645690105155012</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51521,6 +51521,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51743,16 +51752,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51771,14 +51779,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: profile page restriction
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006879FB-6192-4DD0-B157-6CDBD95D8106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6874798B-75B4-4FD0-8E89-E511D5EA4812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>66.645690105155012</v>
+        <v>66.831897001706736</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -17386,11 +17386,11 @@
         <v>4</v>
       </c>
       <c r="E11" s="121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0.12413793103448276</v>
+        <v>0.18620689655172412</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -17406,11 +17406,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="121">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F12" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>6.2068965517241378E-2</v>
+        <v>0.18620689655172412</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -17529,7 +17529,7 @@
       <c r="E18" s="82"/>
       <c r="F18" s="83">
         <f ca="1">SUM(F6:F15)</f>
-        <v>1.3344827586206895</v>
+        <v>1.5206896551724136</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" thickTop="1">
@@ -17697,7 +17697,7 @@
       <c r="E29" s="238"/>
       <c r="F29" s="107">
         <f ca="1">SUM(,F18,F27)</f>
-        <v>1.6344827586206896</v>
+        <v>1.8206896551724137</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23434,11 +23434,11 @@
       </c>
       <c r="D28" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.4086206896551724</v>
+        <v>0.45517241379310341</v>
       </c>
       <c r="E28" s="40">
         <f ca="1">'Settings Page'!F29</f>
-        <v>1.6344827586206896</v>
+        <v>1.8206896551724137</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>66.645690105155012</v>
+        <v>66.831897001706736</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.66645690105155009</v>
+        <v>0.6683189700170673</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>66.645690105155012</v>
+        <v>66.831897001706736</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -51521,15 +51521,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51752,15 +51743,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51779,6 +51771,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
add: favorite-service, add to favorites, favorite videos tab
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27D5800-5124-482E-ACBD-A8157D9BC265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D0898F-C79D-4CCD-AA29-3C94992B1484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>68.304889591939741</v>
+        <v>68.825738005820938</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -11565,11 +11565,11 @@
         <v>2</v>
       </c>
       <c r="E26" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F26" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>7.0129870129870125E-2</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -11585,11 +11585,11 @@
         <v>2</v>
       </c>
       <c r="E27" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F27" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>7.0129870129870125E-2</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -11606,14 +11606,14 @@
       </c>
       <c r="E28" s="80">
         <f>H28*4/I28</f>
-        <v>0</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="F28" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>4.6753246753246748E-2</v>
       </c>
       <c r="H28" s="138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="136">
         <v>3</v>
@@ -11632,11 +11632,11 @@
         <v>1</v>
       </c>
       <c r="E29" s="122">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F29" s="79">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>3.5064935064935063E-2</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -11842,7 +11842,7 @@
       <c r="E39" s="52"/>
       <c r="F39" s="62">
         <f ca="1">SUM(F6:F38)</f>
-        <v>1.7766233766233768</v>
+        <v>1.9987012987012986</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -12001,7 +12001,7 @@
       <c r="E50" s="238"/>
       <c r="F50" s="107">
         <f ca="1">SUM(F39,F48)</f>
-        <v>2.1766233766233767</v>
+        <v>2.3987012987012988</v>
       </c>
     </row>
     <row r="51" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23234,11 +23234,11 @@
       </c>
       <c r="D17" s="41">
         <f t="shared" ref="D17:D38" ca="1" si="0">E17/C17</f>
-        <v>0.66508997182377072</v>
+        <v>0.68998751280737725</v>
       </c>
       <c r="E17" s="40">
         <f ca="1">Components!F55</f>
-        <v>7.9810796618852482</v>
+        <v>8.2798501536885265</v>
       </c>
       <c r="G17" s="42">
         <v>1</v>
@@ -23370,11 +23370,11 @@
       </c>
       <c r="D24" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.54415584415584417</v>
+        <v>0.59967532467532469</v>
       </c>
       <c r="E24" s="40">
         <f ca="1">'Profile Page'!F50</f>
-        <v>2.1766233766233767</v>
+        <v>2.3987012987012988</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>68.304889591939741</v>
+        <v>68.825738005820938</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.68304889591939744</v>
+        <v>0.68825738005820936</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>68.304889591939741</v>
+        <v>68.825738005820938</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -43663,11 +43663,11 @@
         <v>3</v>
       </c>
       <c r="E19" s="53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>0</v>
+        <v>0.29877049180327869</v>
       </c>
       <c r="K19" s="118" t="s">
         <v>68</v>
@@ -44395,7 +44395,7 @@
       <c r="E42" s="52"/>
       <c r="F42" s="62">
         <f ca="1">SUM(F10:F41)</f>
-        <v>5.743032786885248</v>
+        <v>6.0418032786885263</v>
       </c>
     </row>
     <row r="43" spans="2:15" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44535,7 +44535,7 @@
       <c r="E52" s="237"/>
       <c r="F52" s="115">
         <f ca="1">SUM(F42,F50)</f>
-        <v>6.6430327868852483</v>
+        <v>6.9418032786885266</v>
       </c>
     </row>
     <row r="53" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>
@@ -44549,7 +44549,7 @@
       <c r="E55" s="238"/>
       <c r="F55" s="107">
         <f ca="1">SUM(F52,O39)</f>
-        <v>7.9810796618852482</v>
+        <v>8.2798501536885265</v>
       </c>
     </row>
     <row r="56" spans="2:12" ht="15.75" customHeight="1" thickTop="1"/>

</xml_diff>

<commit_message>
add: authLoading for chat page and message sidebar
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D0898F-C79D-4CCD-AA29-3C94992B1484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B63AD8E-B671-4FF5-ACEC-BBFD1A9BF993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="8" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -51521,6 +51521,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51743,16 +51752,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51771,14 +51779,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>

<commit_message>
fix: python file path bug
</commit_message>
<xml_diff>
--- a/Correction Web 25-1 - Final_KN.xlsx
+++ b/Correction Web 25-1 - Final_KN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!_TPA\Web\tpa_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B63AD8E-B671-4FF5-ACEC-BBFD1A9BF993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FEF8840-D7C6-43FE-B509-31A191BF104D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" firstSheet="8" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="51" r:id="rId1"/>
@@ -8048,7 +8048,7 @@
       <c r="A6" s="9"/>
       <c r="B6" s="175">
         <f ca="1">Master!D41</f>
-        <v>68.825738005820938</v>
+        <v>69.21243376928237</v>
       </c>
       <c r="C6" s="176"/>
       <c r="D6" s="176"/>
@@ -17366,11 +17366,11 @@
         <v>10</v>
       </c>
       <c r="E10" s="121">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="2"/>
-        <v>0.15517241379310345</v>
+        <v>0.46551724137931039</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -17529,7 +17529,7 @@
       <c r="E18" s="82"/>
       <c r="F18" s="83">
         <f ca="1">SUM(F6:F15)</f>
-        <v>2.1413793103448273</v>
+        <v>2.4517241379310342</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" thickTop="1">
@@ -17697,7 +17697,7 @@
       <c r="E29" s="238"/>
       <c r="F29" s="107">
         <f ca="1">SUM(,F18,F27)</f>
-        <v>2.4413793103448276</v>
+        <v>2.751724137931034</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -23212,11 +23212,11 @@
       </c>
       <c r="D16" s="41">
         <f ca="1">E16/C16</f>
-        <v>0.79839534883720931</v>
+        <v>0.80618604651162784</v>
       </c>
       <c r="E16" s="40">
         <f ca="1">General!F58</f>
-        <v>15.169511627906976</v>
+        <v>15.31753488372093</v>
       </c>
       <c r="G16" s="98">
         <v>0</v>
@@ -23434,11 +23434,11 @@
       </c>
       <c r="D28" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.6103448275862069</v>
+        <v>0.6879310344827585</v>
       </c>
       <c r="E28" s="40">
         <f ca="1">'Settings Page'!F29</f>
-        <v>2.4413793103448276</v>
+        <v>2.751724137931034</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23498,11 +23498,11 @@
       </c>
       <c r="D32" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.67068345323740997</v>
+        <v>0.67877697841726614</v>
       </c>
       <c r="E32" s="40">
         <f ca="1">'Chat Page'!F45</f>
-        <v>4.69478417266187</v>
+        <v>4.7514388489208628</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -23514,11 +23514,11 @@
       </c>
       <c r="D33" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>0.47230038022813686</v>
+        <v>0.44663498098859317</v>
       </c>
       <c r="E33" s="40">
         <f ca="1">Live!F47</f>
-        <v>2.3615019011406844</v>
+        <v>2.2331749049429659</v>
       </c>
     </row>
     <row r="34" spans="2:16">
@@ -23615,7 +23615,7 @@
       <c r="D39" s="48"/>
       <c r="E39" s="47">
         <f ca="1">SUM(E16:E38)</f>
-        <v>68.825738005820938</v>
+        <v>69.21243376928237</v>
       </c>
     </row>
     <row r="40" spans="2:16" ht="16.5" thickTop="1" thickBot="1">
@@ -23625,7 +23625,7 @@
       <c r="C40" s="203"/>
       <c r="D40" s="205">
         <f ca="1">E39/C39</f>
-        <v>0.68825738005820936</v>
+        <v>0.69212433769282367</v>
       </c>
       <c r="E40" s="203"/>
     </row>
@@ -23636,7 +23636,7 @@
       <c r="C41" s="203"/>
       <c r="D41" s="204">
         <f ca="1">D40 * 100</f>
-        <v>68.825738005820938</v>
+        <v>69.21243376928237</v>
       </c>
       <c r="E41" s="203"/>
     </row>
@@ -24819,11 +24819,11 @@
         <v>5</v>
       </c>
       <c r="E10" s="122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="65">
         <f t="shared" ca="1" si="1"/>
-        <v>0.1133093525179856</v>
+        <v>0.16996402877697842</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -25303,7 +25303,7 @@
       <c r="E34" s="82"/>
       <c r="F34" s="83">
         <f ca="1">SUM(F6:F33)</f>
-        <v>4.1697841726618696</v>
+        <v>4.2264388489208624</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="15.75" thickTop="1">
@@ -25469,7 +25469,7 @@
       <c r="E45" s="238"/>
       <c r="F45" s="107">
         <f ca="1">SUM(F34,F43)</f>
-        <v>4.69478417266187</v>
+        <v>4.7514388489208628</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -26925,11 +26925,11 @@
         <v>15</v>
       </c>
       <c r="E24" s="122">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F24" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0.12832699619771865</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -27181,7 +27181,7 @@
       <c r="E37" s="82"/>
       <c r="F37" s="83">
         <f ca="1">SUM(F7:F36)</f>
-        <v>1.9865019011406846</v>
+        <v>1.8581749049429659</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="15.75" thickTop="1">
@@ -27327,7 +27327,7 @@
       <c r="E47" s="238"/>
       <c r="F47" s="107">
         <f ca="1">SUM(F37,F45)</f>
-        <v>2.3615019011406844</v>
+        <v>2.2331749049429659</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" thickTop="1"/>
@@ -41616,11 +41616,11 @@
         <v>4</v>
       </c>
       <c r="E27" s="131">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" s="25">
         <f t="shared" ca="1" si="1"/>
-        <v>0.29604651162790696</v>
+        <v>0.44406976744186044</v>
       </c>
     </row>
     <row r="28" spans="2:6">
@@ -41695,7 +41695,7 @@
       <c r="E31" s="35"/>
       <c r="F31" s="34">
         <f ca="1">SUM(F6:F30)</f>
-        <v>9.6215116279069761</v>
+        <v>9.7695348837209295</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15.75" thickTop="1"/>
@@ -42131,7 +42131,7 @@
       <c r="E58" s="221"/>
       <c r="F58" s="107">
         <f ca="1">SUM(F31,F45,F56)</f>
-        <v>15.169511627906976</v>
+        <v>15.31753488372093</v>
       </c>
     </row>
     <row r="59" spans="2:6" ht="15.75" customHeight="1" thickTop="1"/>
@@ -51521,15 +51521,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076B14972BA45BD47B3B120E9D54CA4F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="963cb8e90fbbfbeff11449c8f5b5d6a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06dd7198-9f69-4b52-9ad8-623c9ba944b5" xmlns:ns3="1f003750-f5da-409e-99e6-8ff9bea2e38b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="00d017da2f2f45f0e915bbc40802062a" ns2:_="" ns3:_="">
     <xsd:import namespace="06dd7198-9f69-4b52-9ad8-623c9ba944b5"/>
@@ -51752,15 +51743,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{72798FC3-3EF8-485C-8CA8-D899DEC40D90}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51779,6 +51771,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03D307F7-CC51-4BD0-B56F-FB66ABC7A4A5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{3485b963-82ba-4a6f-810f-b5cc226ff898}" enabled="0" method="" siteId="{3485b963-82ba-4a6f-810f-b5cc226ff898}" removed="1"/>

</xml_diff>